<commit_message>
Fix ARES address format and update existing firms
Format house numbers as cisloDomovni/cisloOrientacni (e.g. 788/9 instead of 788 9). Also updated existing firms in firmy.xlsx to match the new format.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/prepis_app/firmy.xlsx
+++ b/prepis_app/firmy.xlsx
@@ -471,7 +471,6 @@
           <t>25101</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -486,7 +485,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Heršpická 788 9, Brno</t>
+          <t>Heršpická 788/9, Brno</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -494,7 +493,6 @@
           <t>63900</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -509,7 +507,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cacovická 1592 30, Brno</t>
+          <t>Cacovická 1592/30, Brno</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -517,7 +515,6 @@
           <t>61400</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -532,7 +529,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Budějovická 1912 64, Praha</t>
+          <t>Budějovická 1912/64, Praha</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -540,7 +537,6 @@
           <t>14000</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -563,7 +559,6 @@
           <t>25101</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -578,7 +573,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hvězdova 1716 2, Praha</t>
+          <t>Hvězdova 1716/2, Praha</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -586,7 +581,6 @@
           <t>14000</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>